<commit_message>
v1.5.0 — Production baseline before asset-light atom recalibration
Captures all incremental improvements since v1.0.1:
- Eval framework (Step 1, 3, 4 benchmarking against internal docs)
- Guidepoint expert library integration (catalog sync + per-analysis agent)
- MECE task framework with 4-gate self-audit, temporal organizing principle
- Atom 11 vs 12 disambiguation (default unstructured for patient-touching)
- Workspace delivery (workbook copied to $PWD after every step)
- Column B protection across all 8 step/eval agents
- API key fallback via shipped data/api_keys.json
- Specificity standard for commentary across all agents
- Labor % expressed as % of revenue (not costs)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/AI Diligence Artifact.xlsx
+++ b/templates/AI Diligence Artifact.xlsx
@@ -1,17 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10714"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amuletcapital.sharepoint.com/sites/Legacy/Shared Documents/General/Admin/AI Initiative/Agentic Strategy (March 2026)/Deliverables/Week 4 (3.26.26)/Agentic Diligence/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/projects/Documents/ai-labor-risk-gp/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="402" documentId="11_F25DC773A252ABDACC1048AF81D87FAC5ADE58EC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A6B509A7-C11D-4C11-A1D6-51948D1AB767}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04CFE304-223F-1A40-9C38-62145E76B78E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="11370" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-    <workbookView minimized="1" xWindow="1480" yWindow="1480" windowWidth="14400" windowHeight="8180" firstSheet="5" activeTab="7" xr2:uid="{5B381CA7-0F59-413C-A7C2-B56F44F5D93B}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30180" windowHeight="17300" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Step 1" sheetId="1" r:id="rId1"/>
@@ -23,7 +22,7 @@
     <sheet name="System Supports Don't Touch &gt;" sheetId="5" r:id="rId7"/>
     <sheet name="Sheet5" sheetId="6" r:id="rId8"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -44,7 +43,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -66,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="123">
   <si>
     <t>AI Diligence Artifact</t>
   </si>
@@ -442,10 +441,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="168" formatCode="_(0.0%_);\(0.0%\);0.0%_)"/>
-    <numFmt numFmtId="169" formatCode="_(0%_);\(0%\);0%_)"/>
-    <numFmt numFmtId="170" formatCode="_(#,##0_);\(#,##0\);_(&quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="171" formatCode="0.0%"/>
+    <numFmt numFmtId="164" formatCode="_(0.0%_);\(0.0%\);0.0%_)"/>
+    <numFmt numFmtId="165" formatCode="_(0%_);\(0%\);0%_)"/>
+    <numFmt numFmtId="166" formatCode="_(#,##0_);\(#,##0\);_(&quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
   <fonts count="14" x14ac:knownFonts="1">
     <font>
@@ -590,7 +589,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -598,22 +597,18 @@
     <xf numFmtId="17" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="17" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -622,13 +617,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="17" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -637,42 +629,34 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="17" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -956,34 +940,34 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:E10"/>
-  <sheetFormatPr defaultRowHeight="10.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="11" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="2.26953125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="9.54296875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="21.1796875" style="1" customWidth="1"/>
-    <col min="4" max="5" width="15.36328125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="1.7265625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="19.26953125" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.7265625" style="1"/>
+    <col min="1" max="1" width="2.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="21.1640625" style="1" customWidth="1"/>
+    <col min="4" max="5" width="15.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="1.6640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:5" ht="13" x14ac:dyDescent="0.15">
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B3" s="7" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B5" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="2:5" ht="12" x14ac:dyDescent="0.4">
-      <c r="B6" s="16" t="s">
+    <row r="6" spans="2:5" ht="14" x14ac:dyDescent="0.3">
+      <c r="B6" s="14" t="s">
         <v>9</v>
       </c>
       <c r="C6" s="4" t="s">
@@ -996,8 +980,8 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B7" s="16">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B7" s="14">
         <v>1</v>
       </c>
       <c r="C7" s="7" t="s">
@@ -1010,8 +994,8 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B8" s="16">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B8" s="14">
         <v>2</v>
       </c>
       <c r="C8" s="7" t="s">
@@ -1024,32 +1008,32 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B9" s="16">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B9" s="14">
         <v>3</v>
       </c>
-      <c r="C9" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="10">
-        <v>0</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B10" s="16">
+      <c r="C9" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="9">
+        <v>0</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B10" s="14">
         <v>4</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="12">
         <f>AVERAGE(D7:D9)</f>
         <v>0</v>
       </c>
-      <c r="E10" s="12"/>
+      <c r="E10" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1058,35 +1042,35 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEEB28C2-D5AF-4724-832E-0D4D205BBD6B}">
-  <dimension ref="B2:E17"/>
-  <sheetFormatPr defaultRowHeight="10.5" x14ac:dyDescent="0.25"/>
+  <dimension ref="B2:E18"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="11" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="2.26953125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="9.54296875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="21.1796875" style="1" customWidth="1"/>
-    <col min="4" max="5" width="15.36328125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="1.7265625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="19.26953125" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.7265625" style="1"/>
+    <col min="1" max="1" width="2.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="21.1640625" style="1" customWidth="1"/>
+    <col min="4" max="5" width="15.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="1.6640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:5" ht="13" x14ac:dyDescent="0.15">
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B3" s="7" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B5" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="2:5" ht="12" x14ac:dyDescent="0.4">
-      <c r="B6" s="16" t="s">
+    <row r="6" spans="2:5" ht="14" x14ac:dyDescent="0.3">
+      <c r="B6" s="14" t="s">
         <v>9</v>
       </c>
       <c r="C6" s="4" t="s">
@@ -1099,11 +1083,11 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B7" s="16">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B7" s="14">
         <v>1</v>
       </c>
-      <c r="C7" s="17">
+      <c r="C7" s="15">
         <v>0</v>
       </c>
       <c r="D7" s="7" t="s">
@@ -1113,11 +1097,11 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B8" s="16">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B8" s="14">
         <v>2</v>
       </c>
-      <c r="C8" s="17">
+      <c r="C8" s="15">
         <v>0</v>
       </c>
       <c r="D8" s="7" t="s">
@@ -1127,137 +1111,152 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B9" s="16">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B9" s="14">
         <v>3</v>
       </c>
-      <c r="C9" s="18">
-        <v>0</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B10" s="16">
+      <c r="C9" s="15">
+        <v>0</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B10" s="14">
         <f>B9+1</f>
         <v>4</v>
       </c>
-      <c r="C10" s="18">
-        <v>0</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="E10" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B11" s="16">
+      <c r="C10" s="15">
+        <v>0</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B11" s="14">
         <f t="shared" ref="B11:B16" si="0">B10+1</f>
         <v>5</v>
       </c>
-      <c r="C11" s="18">
-        <v>0</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="E11" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B12" s="16">
+      <c r="C11" s="15">
+        <v>0</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B12" s="14">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C12" s="18">
-        <v>0</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="E12" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B13" s="16">
+      <c r="C12" s="15">
+        <v>0</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B13" s="14">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C13" s="18">
-        <v>0</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="E13" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B14" s="16">
+      <c r="C13" s="15">
+        <v>0</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B14" s="14">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C14" s="18">
-        <v>0</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B15" s="16">
+      <c r="C14" s="15">
+        <v>0</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B15" s="14">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C15" s="18">
-        <v>0</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B16" s="16">
+      <c r="C15" s="15">
+        <v>0</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B16" s="14">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C16" s="18">
-        <v>0</v>
-      </c>
-      <c r="D16" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="E16" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B17" s="16">
-        <f t="shared" ref="B17" si="1">B16+1</f>
+      <c r="C16" s="15">
+        <v>0</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B17" s="14">
+        <f t="shared" ref="B17:B18" si="1">B16+1</f>
         <v>11</v>
       </c>
-      <c r="C17" s="18">
-        <v>0</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="E17" s="11" t="s">
+      <c r="C17" s="15">
+        <v>0</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B18" s="14">
+        <f t="shared" si="1"/>
+        <v>12</v>
+      </c>
+      <c r="C18" s="15">
+        <v>0</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E18" s="7" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1268,30 +1267,30 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75FAE463-A8E0-417C-9164-24A22BF61796}">
-  <dimension ref="B2:R17"/>
-  <sheetFormatPr defaultRowHeight="10.5" x14ac:dyDescent="0.25"/>
+  <dimension ref="B2:R18"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="11" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="2.26953125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="9.54296875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="21.1796875" style="1" customWidth="1"/>
-    <col min="4" max="15" width="18.54296875" style="1" customWidth="1"/>
-    <col min="16" max="16" width="8.7265625" style="1"/>
-    <col min="17" max="17" width="15.7265625" style="1" customWidth="1"/>
-    <col min="18" max="18" width="19.1796875" style="1" customWidth="1"/>
-    <col min="19" max="16384" width="8.7265625" style="1"/>
+    <col min="1" max="1" width="2.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="21.1640625" style="1" customWidth="1"/>
+    <col min="4" max="15" width="18.5" style="1" customWidth="1"/>
+    <col min="16" max="16" width="8.6640625" style="1"/>
+    <col min="17" max="17" width="15.6640625" style="1" customWidth="1"/>
+    <col min="18" max="18" width="19.1640625" style="1" customWidth="1"/>
+    <col min="19" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:18" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:18" ht="13" x14ac:dyDescent="0.15">
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:18" x14ac:dyDescent="0.15">
       <c r="B3" s="7" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:18" x14ac:dyDescent="0.15">
       <c r="B5" s="3" t="s">
         <v>12</v>
       </c>
@@ -1338,47 +1337,47 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="2:18" ht="35.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B6" s="16" t="s">
+    <row r="6" spans="2:18" ht="35.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="14" t="s">
         <v>9</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="20" t="s">
+      <c r="E6" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="20" t="s">
+      <c r="F6" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="G6" s="20" t="s">
+      <c r="G6" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="H6" s="20" t="s">
+      <c r="H6" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I6" s="20" t="s">
+      <c r="I6" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="J6" s="20" t="s">
+      <c r="J6" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="K6" s="20" t="s">
+      <c r="K6" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="L6" s="20" t="s">
+      <c r="L6" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="M6" s="20" t="s">
+      <c r="M6" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="N6" s="20" t="s">
+      <c r="N6" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="O6" s="20" t="s">
+      <c r="O6" s="17" t="s">
         <v>109</v>
       </c>
       <c r="P6" s="4" t="s">
@@ -1391,11 +1390,11 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B7" s="16">
+    <row r="7" spans="2:18" x14ac:dyDescent="0.15">
+      <c r="B7" s="14">
         <v>1</v>
       </c>
-      <c r="C7" s="19">
+      <c r="C7" s="16">
         <f>'Step 2'!C7</f>
         <v>0</v>
       </c>
@@ -1435,22 +1434,22 @@
       <c r="O7" s="6">
         <v>0</v>
       </c>
-      <c r="P7" s="26" t="str">
+      <c r="P7" s="21" t="str">
         <f>IF(1-SUM(D7:O7)=0,"pass", "fail")</f>
         <v>fail</v>
       </c>
-      <c r="Q7" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="R7" s="21" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B8" s="16">
+      <c r="Q7" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="R7" s="18" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="2:18" x14ac:dyDescent="0.15">
+      <c r="B8" s="14">
         <v>2</v>
       </c>
-      <c r="C8" s="19">
+      <c r="C8" s="16">
         <f>'Step 2'!C8</f>
         <v>0</v>
       </c>
@@ -1490,22 +1489,22 @@
       <c r="O8" s="6">
         <v>0</v>
       </c>
-      <c r="P8" s="26" t="str">
+      <c r="P8" s="21" t="str">
         <f t="shared" ref="P8:P17" si="0">IF(1-SUM(D8:O8)=0,"pass", "fail")</f>
         <v>fail</v>
       </c>
-      <c r="Q8" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="R8" s="21" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B9" s="16">
+      <c r="Q8" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="R8" s="18" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="2:18" x14ac:dyDescent="0.15">
+      <c r="B9" s="14">
         <v>3</v>
       </c>
-      <c r="C9" s="19">
+      <c r="C9" s="16">
         <f>'Step 2'!C9</f>
         <v>0</v>
       </c>
@@ -1545,23 +1544,23 @@
       <c r="O9" s="6">
         <v>0</v>
       </c>
-      <c r="P9" s="26" t="str">
+      <c r="P9" s="21" t="str">
         <f t="shared" si="0"/>
         <v>fail</v>
       </c>
-      <c r="Q9" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="R9" s="22" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B10" s="16">
+      <c r="Q9" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="R9" s="18" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="2:18" x14ac:dyDescent="0.15">
+      <c r="B10" s="14">
         <f>B9+1</f>
         <v>4</v>
       </c>
-      <c r="C10" s="19">
+      <c r="C10" s="16">
         <f>'Step 2'!C10</f>
         <v>0</v>
       </c>
@@ -1601,23 +1600,23 @@
       <c r="O10" s="6">
         <v>0</v>
       </c>
-      <c r="P10" s="26" t="str">
+      <c r="P10" s="21" t="str">
         <f t="shared" si="0"/>
         <v>fail</v>
       </c>
-      <c r="Q10" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="R10" s="22" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B11" s="16">
+      <c r="Q10" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="R10" s="18" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="2:18" x14ac:dyDescent="0.15">
+      <c r="B11" s="14">
         <f t="shared" ref="B11:B16" si="1">B10+1</f>
         <v>5</v>
       </c>
-      <c r="C11" s="19">
+      <c r="C11" s="16">
         <f>'Step 2'!C11</f>
         <v>0</v>
       </c>
@@ -1657,23 +1656,23 @@
       <c r="O11" s="6">
         <v>0</v>
       </c>
-      <c r="P11" s="26" t="str">
+      <c r="P11" s="21" t="str">
         <f t="shared" si="0"/>
         <v>fail</v>
       </c>
-      <c r="Q11" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="R11" s="22" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B12" s="16">
+      <c r="Q11" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="R11" s="18" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="2:18" x14ac:dyDescent="0.15">
+      <c r="B12" s="14">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="C12" s="19">
+      <c r="C12" s="16">
         <f>'Step 2'!C12</f>
         <v>0</v>
       </c>
@@ -1713,23 +1712,23 @@
       <c r="O12" s="6">
         <v>0</v>
       </c>
-      <c r="P12" s="26" t="str">
+      <c r="P12" s="21" t="str">
         <f t="shared" si="0"/>
         <v>fail</v>
       </c>
-      <c r="Q12" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="R12" s="22" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B13" s="16">
+      <c r="Q12" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="R12" s="18" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="2:18" x14ac:dyDescent="0.15">
+      <c r="B13" s="14">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="C13" s="19">
+      <c r="C13" s="16">
         <f>'Step 2'!C13</f>
         <v>0</v>
       </c>
@@ -1769,23 +1768,23 @@
       <c r="O13" s="6">
         <v>0</v>
       </c>
-      <c r="P13" s="26" t="str">
+      <c r="P13" s="21" t="str">
         <f t="shared" si="0"/>
         <v>fail</v>
       </c>
-      <c r="Q13" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="R13" s="22" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="14" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B14" s="16">
+      <c r="Q13" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="R13" s="18" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="2:18" x14ac:dyDescent="0.15">
+      <c r="B14" s="14">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="C14" s="19">
+      <c r="C14" s="16">
         <f>'Step 2'!C14</f>
         <v>0</v>
       </c>
@@ -1825,23 +1824,23 @@
       <c r="O14" s="6">
         <v>0</v>
       </c>
-      <c r="P14" s="26" t="str">
+      <c r="P14" s="21" t="str">
         <f t="shared" si="0"/>
         <v>fail</v>
       </c>
-      <c r="Q14" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="R14" s="22" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B15" s="16">
+      <c r="Q14" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="R14" s="18" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="2:18" x14ac:dyDescent="0.15">
+      <c r="B15" s="14">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="C15" s="19">
+      <c r="C15" s="16">
         <f>'Step 2'!C15</f>
         <v>0</v>
       </c>
@@ -1881,23 +1880,23 @@
       <c r="O15" s="6">
         <v>0</v>
       </c>
-      <c r="P15" s="26" t="str">
+      <c r="P15" s="21" t="str">
         <f t="shared" si="0"/>
         <v>fail</v>
       </c>
-      <c r="Q15" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="R15" s="22" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B16" s="16">
+      <c r="Q15" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="R15" s="18" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="2:18" x14ac:dyDescent="0.15">
+      <c r="B16" s="14">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="C16" s="19">
+      <c r="C16" s="16">
         <f>'Step 2'!C16</f>
         <v>0</v>
       </c>
@@ -1937,22 +1936,22 @@
       <c r="O16" s="6">
         <v>0</v>
       </c>
-      <c r="P16" s="26" t="str">
+      <c r="P16" s="21" t="str">
         <f t="shared" si="0"/>
         <v>fail</v>
       </c>
-      <c r="Q16" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="R16" s="22" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="17" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B17" s="16">
+      <c r="Q16" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="R16" s="18" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="2:18" x14ac:dyDescent="0.15">
+      <c r="B17" s="14">
         <v>11</v>
       </c>
-      <c r="C17" s="19">
+      <c r="C17" s="16">
         <f>'Step 2'!C17</f>
         <v>0</v>
       </c>
@@ -1992,14 +1991,69 @@
       <c r="O17" s="6">
         <v>0</v>
       </c>
-      <c r="P17" s="26" t="str">
+      <c r="P17" s="21" t="str">
         <f t="shared" si="0"/>
         <v>fail</v>
       </c>
-      <c r="Q17" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="R17" s="22" t="s">
+      <c r="Q17" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="R17" s="18" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="2:18" x14ac:dyDescent="0.15">
+      <c r="B18" s="14">
+        <v>12</v>
+      </c>
+      <c r="C18" s="16">
+        <f>'Step 2'!C18</f>
+        <v>0</v>
+      </c>
+      <c r="D18" s="6">
+        <v>0</v>
+      </c>
+      <c r="E18" s="6">
+        <v>0</v>
+      </c>
+      <c r="F18" s="6">
+        <v>0</v>
+      </c>
+      <c r="G18" s="6">
+        <v>0</v>
+      </c>
+      <c r="H18" s="6">
+        <v>0</v>
+      </c>
+      <c r="I18" s="6">
+        <v>0</v>
+      </c>
+      <c r="J18" s="6">
+        <v>0</v>
+      </c>
+      <c r="K18" s="6">
+        <v>0</v>
+      </c>
+      <c r="L18" s="6">
+        <v>0</v>
+      </c>
+      <c r="M18" s="6">
+        <v>0</v>
+      </c>
+      <c r="N18" s="6">
+        <v>0</v>
+      </c>
+      <c r="O18" s="6">
+        <v>0</v>
+      </c>
+      <c r="P18" s="21" t="str">
+        <f t="shared" ref="P18" si="2">IF(1-SUM(D18:O18)=0,"pass", "fail")</f>
+        <v>fail</v>
+      </c>
+      <c r="Q18" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="R18" s="18" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2011,82 +2065,82 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0C1C1C5-6BB7-4202-80DA-FEAE47E837D3}">
   <dimension ref="B2:Q17"/>
-  <sheetFormatPr defaultRowHeight="10.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="11" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="2.26953125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="9.54296875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="21.1796875" style="1" customWidth="1"/>
-    <col min="4" max="14" width="18.54296875" style="1" customWidth="1"/>
-    <col min="15" max="15" width="8.7265625" style="1"/>
-    <col min="16" max="16" width="15.7265625" style="1" customWidth="1"/>
-    <col min="17" max="17" width="19.1796875" style="1" customWidth="1"/>
-    <col min="18" max="16384" width="8.7265625" style="1"/>
+    <col min="1" max="1" width="2.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="21.1640625" style="1" customWidth="1"/>
+    <col min="4" max="14" width="18.5" style="1" customWidth="1"/>
+    <col min="15" max="15" width="8.6640625" style="1"/>
+    <col min="16" max="16" width="15.6640625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="19.1640625" style="1" customWidth="1"/>
+    <col min="18" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:17" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:17" ht="13" x14ac:dyDescent="0.15">
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:17" x14ac:dyDescent="0.15">
       <c r="B3" s="7" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:17" x14ac:dyDescent="0.15">
       <c r="B5" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="2:17" ht="29.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:17" ht="29.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="20" t="str">
+      <c r="C6" s="17" t="str">
         <f>'Step 3'!D6</f>
         <v>1. Information discovery &amp; retrieval</v>
       </c>
-      <c r="D6" s="20" t="str">
+      <c r="D6" s="17" t="str">
         <f>'Step 3'!E6</f>
         <v>2. Extraction &amp; structuring</v>
       </c>
-      <c r="E6" s="20" t="str">
+      <c r="E6" s="17" t="str">
         <f>'Step 3'!F6</f>
         <v>3. Normalization, reconciliation &amp; integration</v>
       </c>
-      <c r="F6" s="20" t="str">
+      <c r="F6" s="17" t="str">
         <f>'Step 3'!G6</f>
         <v>4. Deterministic execution &amp; transaction processing</v>
       </c>
-      <c r="G6" s="20" t="str">
+      <c r="G6" s="17" t="str">
         <f>'Step 3'!H6</f>
         <v>5. Structured triage &amp; decision support</v>
       </c>
-      <c r="H6" s="20" t="str">
+      <c r="H6" s="17" t="str">
         <f>'Step 3'!I6</f>
         <v>6. Authority-bearing judgment &amp; decisioning</v>
       </c>
-      <c r="I6" s="20" t="str">
+      <c r="I6" s="17" t="str">
         <f>'Step 3'!J6</f>
         <v>7. Drafting, synthesis &amp; artifact assembly</v>
       </c>
-      <c r="J6" s="20" t="str">
+      <c r="J6" s="17" t="str">
         <f>'Step 3'!K6</f>
         <v>8. Stakeholder interaction &amp; influence</v>
       </c>
-      <c r="K6" s="20" t="str">
+      <c r="K6" s="17" t="str">
         <f>'Step 3'!L6</f>
         <v>9. Workflow orchestration &amp; exception resolution</v>
       </c>
-      <c r="L6" s="20" t="str">
+      <c r="L6" s="17" t="str">
         <f>'Step 3'!M6</f>
         <v>10. Assurance, compliance &amp; traceability</v>
       </c>
-      <c r="M6" s="20" t="str">
+      <c r="M6" s="17" t="str">
         <f>'Step 3'!N6</f>
         <v>11. Physical execution - Structured / Predictable</v>
       </c>
-      <c r="N6" s="20" t="str">
+      <c r="N6" s="17" t="str">
         <f>'Step 3'!O6</f>
         <v>12. Physical execution - Variable/unstructured</v>
       </c>
@@ -2094,269 +2148,269 @@
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
     </row>
-    <row r="7" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B7" s="16" t="str" cm="1">
+    <row r="7" spans="2:17" x14ac:dyDescent="0.15">
+      <c r="B7" s="14" t="str" cm="1">
         <f t="array" ref="B7:B12">TRANSPOSE(Sheet5!B1:G1)</f>
         <v>Today Low</v>
       </c>
-      <c r="C7" s="25" cm="1">
+      <c r="C7" s="20" cm="1">
         <f t="array" ref="C7:N12">TRANSPOSE(Sheet5!B2:G13)</f>
         <v>0.4</v>
       </c>
-      <c r="D7" s="25">
+      <c r="D7" s="20">
         <v>0.45</v>
       </c>
-      <c r="E7" s="25">
+      <c r="E7" s="20">
         <v>0.25</v>
       </c>
-      <c r="F7" s="25">
+      <c r="F7" s="20">
         <v>0.4</v>
       </c>
-      <c r="G7" s="25">
+      <c r="G7" s="20">
         <v>0.4</v>
       </c>
-      <c r="H7" s="25">
+      <c r="H7" s="20">
         <v>0.1</v>
       </c>
-      <c r="I7" s="25">
+      <c r="I7" s="20">
         <v>0.4</v>
       </c>
-      <c r="J7" s="25">
+      <c r="J7" s="20">
         <v>0.1</v>
       </c>
-      <c r="K7" s="25">
+      <c r="K7" s="20">
         <v>0.15</v>
       </c>
-      <c r="L7" s="25">
+      <c r="L7" s="20">
         <v>0.2</v>
       </c>
-      <c r="M7" s="25">
+      <c r="M7" s="20">
         <v>0.45</v>
       </c>
-      <c r="N7" s="25">
+      <c r="N7" s="20">
         <v>0.05</v>
       </c>
-      <c r="P7" s="21"/>
-      <c r="Q7" s="21"/>
-    </row>
-    <row r="8" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B8" s="16" t="str">
+      <c r="P7" s="18"/>
+      <c r="Q7" s="18"/>
+    </row>
+    <row r="8" spans="2:17" x14ac:dyDescent="0.15">
+      <c r="B8" s="14" t="str">
         <v>Today High</v>
       </c>
-      <c r="C8" s="25">
+      <c r="C8" s="20">
         <v>0.65</v>
       </c>
-      <c r="D8" s="25">
+      <c r="D8" s="20">
         <v>0.75</v>
       </c>
-      <c r="E8" s="25">
+      <c r="E8" s="20">
         <v>0.55000000000000004</v>
       </c>
-      <c r="F8" s="25">
+      <c r="F8" s="20">
         <v>0.7</v>
       </c>
-      <c r="G8" s="25">
+      <c r="G8" s="20">
         <v>0.7</v>
       </c>
-      <c r="H8" s="25">
+      <c r="H8" s="20">
         <v>0.25</v>
       </c>
-      <c r="I8" s="25">
+      <c r="I8" s="20">
         <v>0.7</v>
       </c>
-      <c r="J8" s="25">
+      <c r="J8" s="20">
         <v>0.45</v>
       </c>
-      <c r="K8" s="25">
+      <c r="K8" s="20">
         <v>0.4</v>
       </c>
-      <c r="L8" s="25">
+      <c r="L8" s="20">
         <v>0.45</v>
       </c>
-      <c r="M8" s="25">
+      <c r="M8" s="20">
         <v>0.75</v>
       </c>
-      <c r="N8" s="25">
+      <c r="N8" s="20">
         <v>0.15</v>
       </c>
-      <c r="P8" s="21"/>
-      <c r="Q8" s="21"/>
-    </row>
-    <row r="9" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B9" s="16" t="str">
+      <c r="P8" s="18"/>
+      <c r="Q8" s="18"/>
+    </row>
+    <row r="9" spans="2:17" x14ac:dyDescent="0.15">
+      <c r="B9" s="14" t="str">
         <v>2–3y Low</v>
       </c>
-      <c r="C9" s="25">
+      <c r="C9" s="20">
         <v>0.6</v>
       </c>
-      <c r="D9" s="25">
+      <c r="D9" s="20">
         <v>0.65</v>
       </c>
-      <c r="E9" s="25">
+      <c r="E9" s="20">
         <v>0.45</v>
       </c>
-      <c r="F9" s="25">
+      <c r="F9" s="20">
         <v>0.55000000000000004</v>
       </c>
-      <c r="G9" s="25">
+      <c r="G9" s="20">
         <v>0.55000000000000004</v>
       </c>
-      <c r="H9" s="25">
+      <c r="H9" s="20">
         <v>0.2</v>
       </c>
-      <c r="I9" s="25">
+      <c r="I9" s="20">
         <v>0.6</v>
       </c>
-      <c r="J9" s="25">
+      <c r="J9" s="20">
         <v>0.2</v>
       </c>
-      <c r="K9" s="25">
+      <c r="K9" s="20">
         <v>0.35</v>
       </c>
-      <c r="L9" s="25">
+      <c r="L9" s="20">
         <v>0.3</v>
       </c>
-      <c r="M9" s="25">
+      <c r="M9" s="20">
         <v>0.6</v>
       </c>
-      <c r="N9" s="25">
+      <c r="N9" s="20">
         <v>0.1</v>
       </c>
-      <c r="P9" s="22"/>
-      <c r="Q9" s="22"/>
-    </row>
-    <row r="10" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B10" s="16" t="str">
+      <c r="P9" s="18"/>
+      <c r="Q9" s="18"/>
+    </row>
+    <row r="10" spans="2:17" x14ac:dyDescent="0.15">
+      <c r="B10" s="14" t="str">
         <v>2–3y High</v>
       </c>
-      <c r="C10" s="25">
+      <c r="C10" s="20">
         <v>0.85</v>
       </c>
-      <c r="D10" s="25">
+      <c r="D10" s="20">
         <v>0.9</v>
       </c>
-      <c r="E10" s="25">
+      <c r="E10" s="20">
         <v>0.75</v>
       </c>
-      <c r="F10" s="25">
+      <c r="F10" s="20">
         <v>0.85</v>
       </c>
-      <c r="G10" s="25">
+      <c r="G10" s="20">
         <v>0.85</v>
       </c>
-      <c r="H10" s="25">
+      <c r="H10" s="20">
         <v>0.45</v>
       </c>
-      <c r="I10" s="25">
+      <c r="I10" s="20">
         <v>0.85</v>
       </c>
-      <c r="J10" s="25">
+      <c r="J10" s="20">
         <v>0.6</v>
       </c>
-      <c r="K10" s="25">
+      <c r="K10" s="20">
         <v>0.65</v>
       </c>
-      <c r="L10" s="25">
+      <c r="L10" s="20">
         <v>0.6</v>
       </c>
-      <c r="M10" s="25">
+      <c r="M10" s="20">
         <v>0.85</v>
       </c>
-      <c r="N10" s="25">
+      <c r="N10" s="20">
         <v>0.25</v>
       </c>
-      <c r="P10" s="22"/>
-      <c r="Q10" s="22"/>
-    </row>
-    <row r="11" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B11" s="16" t="str">
+      <c r="P10" s="18"/>
+      <c r="Q10" s="18"/>
+    </row>
+    <row r="11" spans="2:17" x14ac:dyDescent="0.15">
+      <c r="B11" s="14" t="str">
         <v>5–10y Low</v>
       </c>
-      <c r="C11" s="25">
+      <c r="C11" s="20">
         <v>0.75</v>
       </c>
-      <c r="D11" s="25">
+      <c r="D11" s="20">
         <v>0.8</v>
       </c>
-      <c r="E11" s="25">
+      <c r="E11" s="20">
         <v>0.6</v>
       </c>
-      <c r="F11" s="25">
+      <c r="F11" s="20">
         <v>0.75</v>
       </c>
-      <c r="G11" s="25">
+      <c r="G11" s="20">
         <v>0.7</v>
       </c>
-      <c r="H11" s="25">
+      <c r="H11" s="20">
         <v>0.35</v>
       </c>
-      <c r="I11" s="25">
+      <c r="I11" s="20">
         <v>0.75</v>
       </c>
-      <c r="J11" s="25">
+      <c r="J11" s="20">
         <v>0.35</v>
       </c>
-      <c r="K11" s="25">
+      <c r="K11" s="20">
         <v>0.55000000000000004</v>
       </c>
-      <c r="L11" s="25">
+      <c r="L11" s="20">
         <v>0.45</v>
       </c>
-      <c r="M11" s="25">
+      <c r="M11" s="20">
         <v>0.75</v>
       </c>
-      <c r="N11" s="25">
+      <c r="N11" s="20">
         <v>0.2</v>
       </c>
-      <c r="P11" s="22"/>
-      <c r="Q11" s="22"/>
-    </row>
-    <row r="12" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B12" s="16" t="str">
+      <c r="P11" s="18"/>
+      <c r="Q11" s="18"/>
+    </row>
+    <row r="12" spans="2:17" x14ac:dyDescent="0.15">
+      <c r="B12" s="14" t="str">
         <v>5–10y High</v>
       </c>
-      <c r="C12" s="25">
+      <c r="C12" s="20">
         <v>0.95</v>
       </c>
-      <c r="D12" s="25">
+      <c r="D12" s="20">
         <v>0.97</v>
       </c>
-      <c r="E12" s="25">
+      <c r="E12" s="20">
         <v>0.9</v>
       </c>
-      <c r="F12" s="25">
+      <c r="F12" s="20">
         <v>0.95</v>
       </c>
-      <c r="G12" s="25">
+      <c r="G12" s="20">
         <v>0.95</v>
       </c>
-      <c r="H12" s="25">
+      <c r="H12" s="20">
         <v>0.65</v>
       </c>
-      <c r="I12" s="25">
+      <c r="I12" s="20">
         <v>0.95</v>
       </c>
-      <c r="J12" s="25">
+      <c r="J12" s="20">
         <v>0.8</v>
       </c>
-      <c r="K12" s="25">
+      <c r="K12" s="20">
         <v>0.85</v>
       </c>
-      <c r="L12" s="25">
+      <c r="L12" s="20">
         <v>0.75</v>
       </c>
-      <c r="M12" s="25">
+      <c r="M12" s="20">
         <v>0.95</v>
       </c>
-      <c r="N12" s="25">
+      <c r="N12" s="20">
         <v>0.45</v>
       </c>
-      <c r="P12" s="22"/>
-      <c r="Q12" s="22"/>
-    </row>
-    <row r="13" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B13" s="16"/>
-      <c r="C13" s="19"/>
+      <c r="P12" s="18"/>
+      <c r="Q12" s="18"/>
+    </row>
+    <row r="13" spans="2:17" x14ac:dyDescent="0.15">
+      <c r="B13" s="14"/>
+      <c r="C13" s="16"/>
       <c r="D13" s="6"/>
       <c r="E13" s="6"/>
       <c r="F13" s="6"/>
@@ -2368,12 +2422,12 @@
       <c r="L13" s="6"/>
       <c r="M13" s="6"/>
       <c r="N13" s="6"/>
-      <c r="P13" s="22"/>
-      <c r="Q13" s="22"/>
-    </row>
-    <row r="14" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B14" s="16"/>
-      <c r="C14" s="19"/>
+      <c r="P13" s="18"/>
+      <c r="Q13" s="18"/>
+    </row>
+    <row r="14" spans="2:17" x14ac:dyDescent="0.15">
+      <c r="B14" s="14"/>
+      <c r="C14" s="16"/>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
       <c r="F14" s="6"/>
@@ -2385,12 +2439,12 @@
       <c r="L14" s="6"/>
       <c r="M14" s="6"/>
       <c r="N14" s="6"/>
-      <c r="P14" s="22"/>
-      <c r="Q14" s="22"/>
-    </row>
-    <row r="15" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B15" s="16"/>
-      <c r="C15" s="19"/>
+      <c r="P14" s="18"/>
+      <c r="Q14" s="18"/>
+    </row>
+    <row r="15" spans="2:17" x14ac:dyDescent="0.15">
+      <c r="B15" s="14"/>
+      <c r="C15" s="16"/>
       <c r="D15" s="6"/>
       <c r="E15" s="6"/>
       <c r="F15" s="6"/>
@@ -2402,12 +2456,12 @@
       <c r="L15" s="6"/>
       <c r="M15" s="6"/>
       <c r="N15" s="6"/>
-      <c r="P15" s="22"/>
-      <c r="Q15" s="22"/>
-    </row>
-    <row r="16" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B16" s="16"/>
-      <c r="C16" s="19"/>
+      <c r="P15" s="18"/>
+      <c r="Q15" s="18"/>
+    </row>
+    <row r="16" spans="2:17" x14ac:dyDescent="0.15">
+      <c r="B16" s="14"/>
+      <c r="C16" s="16"/>
       <c r="D16" s="6"/>
       <c r="E16" s="6"/>
       <c r="F16" s="6"/>
@@ -2419,12 +2473,12 @@
       <c r="L16" s="6"/>
       <c r="M16" s="6"/>
       <c r="N16" s="6"/>
-      <c r="P16" s="22"/>
-      <c r="Q16" s="22"/>
-    </row>
-    <row r="17" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B17" s="16"/>
-      <c r="C17" s="19"/>
+      <c r="P16" s="18"/>
+      <c r="Q16" s="18"/>
+    </row>
+    <row r="17" spans="2:17" x14ac:dyDescent="0.15">
+      <c r="B17" s="14"/>
+      <c r="C17" s="16"/>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
       <c r="F17" s="6"/>
@@ -2436,8 +2490,8 @@
       <c r="L17" s="6"/>
       <c r="M17" s="6"/>
       <c r="N17" s="6"/>
-      <c r="P17" s="22"/>
-      <c r="Q17" s="22"/>
+      <c r="P17" s="18"/>
+      <c r="Q17" s="18"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2447,28 +2501,28 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3934178E-90C5-436E-957E-8832BEB865EC}">
   <dimension ref="B2:S21"/>
-  <sheetFormatPr defaultRowHeight="10.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="11" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="2.26953125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="9.54296875" style="1" customWidth="1"/>
-    <col min="3" max="4" width="21.1796875" style="1" customWidth="1"/>
-    <col min="5" max="6" width="15.36328125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="1.7265625" style="1" customWidth="1"/>
-    <col min="8" max="19" width="14.90625" style="1" customWidth="1"/>
-    <col min="20" max="16384" width="8.7265625" style="1"/>
+    <col min="1" max="1" width="2.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5" style="1" customWidth="1"/>
+    <col min="3" max="4" width="21.1640625" style="1" customWidth="1"/>
+    <col min="5" max="6" width="15.33203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="1.6640625" style="1" customWidth="1"/>
+    <col min="8" max="19" width="14.83203125" style="1" customWidth="1"/>
+    <col min="20" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:19" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:19" ht="13" x14ac:dyDescent="0.15">
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:19" x14ac:dyDescent="0.15">
       <c r="B3" s="7" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:19" x14ac:dyDescent="0.15">
       <c r="B5" s="3" t="s">
         <v>110</v>
       </c>
@@ -2524,8 +2578,8 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="6" spans="2:19" ht="32" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B6" s="16" t="s">
+    <row r="6" spans="2:19" ht="32" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="14" t="s">
         <v>9</v>
       </c>
       <c r="C6" s="4" t="s">
@@ -2540,60 +2594,60 @@
       <c r="F6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="H6" s="30" t="str">
+      <c r="H6" s="24" t="str">
         <f>'Appendix A'!C6</f>
         <v>1. Information discovery &amp; retrieval</v>
       </c>
-      <c r="I6" s="30" t="str">
+      <c r="I6" s="24" t="str">
         <f>'Appendix A'!D6</f>
         <v>2. Extraction &amp; structuring</v>
       </c>
-      <c r="J6" s="30" t="str">
+      <c r="J6" s="24" t="str">
         <f>'Appendix A'!E6</f>
         <v>3. Normalization, reconciliation &amp; integration</v>
       </c>
-      <c r="K6" s="30" t="str">
+      <c r="K6" s="24" t="str">
         <f>'Appendix A'!F6</f>
         <v>4. Deterministic execution &amp; transaction processing</v>
       </c>
-      <c r="L6" s="30" t="str">
+      <c r="L6" s="24" t="str">
         <f>'Appendix A'!G6</f>
         <v>5. Structured triage &amp; decision support</v>
       </c>
-      <c r="M6" s="30" t="str">
+      <c r="M6" s="24" t="str">
         <f>'Appendix A'!H6</f>
         <v>6. Authority-bearing judgment &amp; decisioning</v>
       </c>
-      <c r="N6" s="30" t="str">
+      <c r="N6" s="24" t="str">
         <f>'Appendix A'!I6</f>
         <v>7. Drafting, synthesis &amp; artifact assembly</v>
       </c>
-      <c r="O6" s="30" t="str">
+      <c r="O6" s="24" t="str">
         <f>'Appendix A'!J6</f>
         <v>8. Stakeholder interaction &amp; influence</v>
       </c>
-      <c r="P6" s="30" t="str">
+      <c r="P6" s="24" t="str">
         <f>'Appendix A'!K6</f>
         <v>9. Workflow orchestration &amp; exception resolution</v>
       </c>
-      <c r="Q6" s="30" t="str">
+      <c r="Q6" s="24" t="str">
         <f>'Appendix A'!L6</f>
         <v>10. Assurance, compliance &amp; traceability</v>
       </c>
-      <c r="R6" s="30" t="str">
+      <c r="R6" s="24" t="str">
         <f>'Appendix A'!M6</f>
         <v>11. Physical execution - Structured / Predictable</v>
       </c>
-      <c r="S6" s="30" t="str">
+      <c r="S6" s="24" t="str">
         <f>'Appendix A'!N6</f>
         <v>12. Physical execution - Variable/unstructured</v>
       </c>
     </row>
-    <row r="7" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B7" s="16">
+    <row r="7" spans="2:19" x14ac:dyDescent="0.15">
+      <c r="B7" s="14">
         <v>1</v>
       </c>
-      <c r="C7" s="29">
+      <c r="C7" s="23">
         <f>'Step 3'!C7</f>
         <v>0</v>
       </c>
@@ -2655,11 +2709,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B8" s="16">
+    <row r="8" spans="2:19" x14ac:dyDescent="0.15">
+      <c r="B8" s="14">
         <v>2</v>
       </c>
-      <c r="C8" s="29">
+      <c r="C8" s="23">
         <f>'Step 3'!C8</f>
         <v>0</v>
       </c>
@@ -2721,21 +2775,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="16">
+    <row r="9" spans="2:19" x14ac:dyDescent="0.15">
+      <c r="B9" s="14">
         <v>3</v>
       </c>
-      <c r="C9" s="29">
+      <c r="C9" s="23">
         <f>'Step 3'!C9</f>
         <v>0</v>
       </c>
-      <c r="D9" s="27">
-        <v>0</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F9" s="11" t="s">
+      <c r="D9" s="8">
+        <v>0</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="F9" s="7" t="s">
         <v>6</v>
       </c>
       <c r="H9" s="5">
@@ -2787,22 +2841,22 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="16">
+    <row r="10" spans="2:19" x14ac:dyDescent="0.15">
+      <c r="B10" s="14">
         <f>B9+1</f>
         <v>4</v>
       </c>
-      <c r="C10" s="29">
+      <c r="C10" s="23">
         <f>'Step 3'!C10</f>
         <v>0</v>
       </c>
-      <c r="D10" s="27">
-        <v>0</v>
-      </c>
-      <c r="E10" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F10" s="11" t="s">
+      <c r="D10" s="8">
+        <v>0</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="F10" s="7" t="s">
         <v>6</v>
       </c>
       <c r="H10" s="5">
@@ -2854,22 +2908,22 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="16">
-        <f t="shared" ref="B11:B17" si="0">B10+1</f>
+    <row r="11" spans="2:19" x14ac:dyDescent="0.15">
+      <c r="B11" s="14">
+        <f t="shared" ref="B11:B18" si="0">B10+1</f>
         <v>5</v>
       </c>
-      <c r="C11" s="29">
+      <c r="C11" s="23">
         <f>'Step 3'!C11</f>
         <v>0</v>
       </c>
-      <c r="D11" s="27">
-        <v>0</v>
-      </c>
-      <c r="E11" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F11" s="11" t="s">
+      <c r="D11" s="8">
+        <v>0</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="F11" s="7" t="s">
         <v>6</v>
       </c>
       <c r="H11" s="5">
@@ -2921,22 +2975,22 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B12" s="16">
+    <row r="12" spans="2:19" x14ac:dyDescent="0.15">
+      <c r="B12" s="14">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C12" s="29">
+      <c r="C12" s="23">
         <f>'Step 3'!C12</f>
         <v>0</v>
       </c>
-      <c r="D12" s="27">
-        <v>0</v>
-      </c>
-      <c r="E12" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F12" s="11" t="s">
+      <c r="D12" s="8">
+        <v>0</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="F12" s="7" t="s">
         <v>6</v>
       </c>
       <c r="H12" s="5">
@@ -2988,22 +3042,22 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B13" s="16">
+    <row r="13" spans="2:19" x14ac:dyDescent="0.15">
+      <c r="B13" s="14">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C13" s="29">
+      <c r="C13" s="23">
         <f>'Step 3'!C13</f>
         <v>0</v>
       </c>
-      <c r="D13" s="27">
-        <v>0</v>
-      </c>
-      <c r="E13" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F13" s="11" t="s">
+      <c r="D13" s="8">
+        <v>0</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="F13" s="7" t="s">
         <v>6</v>
       </c>
       <c r="H13" s="5">
@@ -3055,22 +3109,22 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B14" s="16">
+    <row r="14" spans="2:19" x14ac:dyDescent="0.15">
+      <c r="B14" s="14">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C14" s="29">
+      <c r="C14" s="23">
         <f>'Step 3'!C14</f>
         <v>0</v>
       </c>
-      <c r="D14" s="27">
-        <v>0</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F14" s="11" t="s">
+      <c r="D14" s="8">
+        <v>0</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="F14" s="7" t="s">
         <v>6</v>
       </c>
       <c r="H14" s="5">
@@ -3122,22 +3176,22 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B15" s="16">
+    <row r="15" spans="2:19" x14ac:dyDescent="0.15">
+      <c r="B15" s="14">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C15" s="29">
+      <c r="C15" s="23">
         <f>'Step 3'!C15</f>
         <v>0</v>
       </c>
-      <c r="D15" s="27">
-        <v>0</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F15" s="11" t="s">
+      <c r="D15" s="8">
+        <v>0</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="F15" s="7" t="s">
         <v>6</v>
       </c>
       <c r="H15" s="5">
@@ -3189,22 +3243,22 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B16" s="16">
+    <row r="16" spans="2:19" x14ac:dyDescent="0.15">
+      <c r="B16" s="14">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C16" s="29">
+      <c r="C16" s="23">
         <f>'Step 3'!C16</f>
         <v>0</v>
       </c>
-      <c r="D16" s="27">
-        <v>0</v>
-      </c>
-      <c r="E16" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F16" s="11" t="s">
+      <c r="D16" s="8">
+        <v>0</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="F16" s="7" t="s">
         <v>6</v>
       </c>
       <c r="H16" s="5">
@@ -3256,22 +3310,22 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="16">
+    <row r="17" spans="2:19" x14ac:dyDescent="0.15">
+      <c r="B17" s="14">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C17" s="29">
+      <c r="C17" s="23">
         <f>'Step 3'!C17</f>
         <v>0</v>
       </c>
-      <c r="D17" s="27">
-        <v>0</v>
-      </c>
-      <c r="E17" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F17" s="11" t="s">
+      <c r="D17" s="8">
+        <v>0</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="F17" s="7" t="s">
         <v>6</v>
       </c>
       <c r="H17" s="5">
@@ -3323,7 +3377,74 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:19" x14ac:dyDescent="0.15">
+      <c r="B18" s="14">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="C18" s="23">
+        <f>'Step 3'!C18</f>
+        <v>0</v>
+      </c>
+      <c r="D18" s="8">
+        <v>0</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H18" s="5">
+        <f>H$5*'Step 3'!D18</f>
+        <v>0</v>
+      </c>
+      <c r="I18" s="5">
+        <f>I$5*'Step 3'!E18</f>
+        <v>0</v>
+      </c>
+      <c r="J18" s="5">
+        <f>J$5*'Step 3'!F18</f>
+        <v>0</v>
+      </c>
+      <c r="K18" s="5">
+        <f>K$5*'Step 3'!G18</f>
+        <v>0</v>
+      </c>
+      <c r="L18" s="5">
+        <f>L$5*'Step 3'!H18</f>
+        <v>0</v>
+      </c>
+      <c r="M18" s="5">
+        <f>M$5*'Step 3'!I18</f>
+        <v>0</v>
+      </c>
+      <c r="N18" s="5">
+        <f>N$5*'Step 3'!J18</f>
+        <v>0</v>
+      </c>
+      <c r="O18" s="5">
+        <f>O$5*'Step 3'!K18</f>
+        <v>0</v>
+      </c>
+      <c r="P18" s="5">
+        <f>P$5*'Step 3'!L18</f>
+        <v>0</v>
+      </c>
+      <c r="Q18" s="5">
+        <f>Q$5*'Step 3'!M18</f>
+        <v>0</v>
+      </c>
+      <c r="R18" s="5">
+        <f>R$5*'Step 3'!N18</f>
+        <v>0</v>
+      </c>
+      <c r="S18" s="5">
+        <f>S$5*'Step 3'!O18</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="2:19" x14ac:dyDescent="0.15">
       <c r="B21" s="1" t="s">
         <v>112</v>
       </c>
@@ -3351,312 +3472,336 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DE691CC-5343-4530-A59A-32E9FBAB9B75}">
   <dimension ref="B2:H27"/>
-  <sheetFormatPr defaultRowHeight="10.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="11" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="2.26953125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="9.54296875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="21.1796875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="15.36328125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="19.7265625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="1.7265625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="19.26953125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="17.6328125" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="8.7265625" style="1"/>
+    <col min="1" max="1" width="2.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="21.1640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="19.6640625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="1.6640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="17.6640625" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:8" ht="13" x14ac:dyDescent="0.15">
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:8" x14ac:dyDescent="0.15">
       <c r="B3" s="7" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="2:8" ht="12" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:8" ht="14" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="15" t="s">
+      <c r="D6" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="E6" s="15" t="str">
+      <c r="E6" s="13" t="str">
         <f>_xlfn.CONCAT("% of Labor '",'Step 4 Weighted Calc'!C21, "' Case")</f>
         <v>% of Labor 'Today Low' Case</v>
       </c>
-      <c r="G6" s="15" t="s">
+      <c r="G6" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="H6" s="15" t="s">
+      <c r="H6" s="13" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B7" s="16">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.15">
+      <c r="B7" s="14">
         <v>1</v>
       </c>
-      <c r="C7" s="28">
+      <c r="C7" s="22">
         <f>'Step 2'!C7</f>
         <v>0</v>
       </c>
-      <c r="D7" s="31">
+      <c r="D7" s="25">
         <f>'Step 4 Weighted Calc'!D7</f>
         <v>0</v>
       </c>
-      <c r="E7" s="31">
+      <c r="E7" s="25">
         <f>'Step 4 Weighted Calc'!D7*SUM('Step 4 Weighted Calc'!H7:S7)</f>
         <v>0</v>
       </c>
-      <c r="G7" s="21" t="s">
-        <v>6</v>
-      </c>
-      <c r="H7" s="21" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="16">
+      <c r="G7" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="H7" s="18" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.15">
+      <c r="B8" s="14">
         <v>2</v>
       </c>
-      <c r="C8" s="28">
+      <c r="C8" s="22">
         <f>'Step 2'!C8</f>
         <v>0</v>
       </c>
-      <c r="D8" s="31">
+      <c r="D8" s="25">
         <f>'Step 4 Weighted Calc'!D8</f>
         <v>0</v>
       </c>
-      <c r="E8" s="31">
+      <c r="E8" s="25">
         <f>'Step 4 Weighted Calc'!D8*SUM('Step 4 Weighted Calc'!H8:S8)</f>
         <v>0</v>
       </c>
-      <c r="G8" s="21" t="s">
-        <v>6</v>
-      </c>
-      <c r="H8" s="21" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B9" s="16">
+      <c r="G8" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="H8" s="18" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.15">
+      <c r="B9" s="14">
         <v>3</v>
       </c>
-      <c r="C9" s="28">
+      <c r="C9" s="22">
         <f>'Step 2'!C9</f>
         <v>0</v>
       </c>
-      <c r="D9" s="31">
+      <c r="D9" s="25">
         <f>'Step 4 Weighted Calc'!D9</f>
         <v>0</v>
       </c>
-      <c r="E9" s="31">
+      <c r="E9" s="25">
         <f>'Step 4 Weighted Calc'!D9*SUM('Step 4 Weighted Calc'!H9:S9)</f>
         <v>0</v>
       </c>
-      <c r="G9" s="21" t="s">
-        <v>6</v>
-      </c>
-      <c r="H9" s="21" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B10" s="16">
+      <c r="G9" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="H9" s="18" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.15">
+      <c r="B10" s="14">
         <f>B9+1</f>
         <v>4</v>
       </c>
-      <c r="C10" s="28">
+      <c r="C10" s="22">
         <f>'Step 2'!C10</f>
         <v>0</v>
       </c>
-      <c r="D10" s="31">
+      <c r="D10" s="25">
         <f>'Step 4 Weighted Calc'!D10</f>
         <v>0</v>
       </c>
-      <c r="E10" s="31">
+      <c r="E10" s="25">
         <f>'Step 4 Weighted Calc'!D10*SUM('Step 4 Weighted Calc'!H10:S10)</f>
         <v>0</v>
       </c>
-      <c r="G10" s="21" t="s">
-        <v>6</v>
-      </c>
-      <c r="H10" s="21" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B11" s="16">
-        <f t="shared" ref="B11:B17" si="0">B10+1</f>
+      <c r="G10" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="H10" s="18" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.15">
+      <c r="B11" s="14">
+        <f t="shared" ref="B11:B18" si="0">B10+1</f>
         <v>5</v>
       </c>
-      <c r="C11" s="28">
+      <c r="C11" s="22">
         <f>'Step 2'!C11</f>
         <v>0</v>
       </c>
-      <c r="D11" s="31">
+      <c r="D11" s="25">
         <f>'Step 4 Weighted Calc'!D11</f>
         <v>0</v>
       </c>
-      <c r="E11" s="31">
+      <c r="E11" s="25">
         <f>'Step 4 Weighted Calc'!D11*SUM('Step 4 Weighted Calc'!H11:S11)</f>
         <v>0</v>
       </c>
-      <c r="G11" s="21" t="s">
-        <v>6</v>
-      </c>
-      <c r="H11" s="21" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B12" s="16">
+      <c r="G11" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="H11" s="18" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.15">
+      <c r="B12" s="14">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C12" s="28">
+      <c r="C12" s="22">
         <f>'Step 2'!C12</f>
         <v>0</v>
       </c>
-      <c r="D12" s="31">
+      <c r="D12" s="25">
         <f>'Step 4 Weighted Calc'!D12</f>
         <v>0</v>
       </c>
-      <c r="E12" s="31">
+      <c r="E12" s="25">
         <f>'Step 4 Weighted Calc'!D12*SUM('Step 4 Weighted Calc'!H12:S12)</f>
         <v>0</v>
       </c>
-      <c r="G12" s="21" t="s">
-        <v>6</v>
-      </c>
-      <c r="H12" s="21" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B13" s="16">
+      <c r="G12" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="H12" s="18" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.15">
+      <c r="B13" s="14">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C13" s="28">
+      <c r="C13" s="22">
         <f>'Step 2'!C13</f>
         <v>0</v>
       </c>
-      <c r="D13" s="31">
+      <c r="D13" s="25">
         <f>'Step 4 Weighted Calc'!D13</f>
         <v>0</v>
       </c>
-      <c r="E13" s="31">
+      <c r="E13" s="25">
         <f>'Step 4 Weighted Calc'!D13*SUM('Step 4 Weighted Calc'!H13:S13)</f>
         <v>0</v>
       </c>
-      <c r="G13" s="21" t="s">
-        <v>6</v>
-      </c>
-      <c r="H13" s="21" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B14" s="16">
+      <c r="G13" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="H13" s="18" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" x14ac:dyDescent="0.15">
+      <c r="B14" s="14">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C14" s="28">
+      <c r="C14" s="22">
         <f>'Step 2'!C14</f>
         <v>0</v>
       </c>
-      <c r="D14" s="31">
+      <c r="D14" s="25">
         <f>'Step 4 Weighted Calc'!D14</f>
         <v>0</v>
       </c>
-      <c r="E14" s="31">
+      <c r="E14" s="25">
         <f>'Step 4 Weighted Calc'!D14*SUM('Step 4 Weighted Calc'!H14:S14)</f>
         <v>0</v>
       </c>
-      <c r="G14" s="21" t="s">
-        <v>6</v>
-      </c>
-      <c r="H14" s="21" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B15" s="16">
+      <c r="G14" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="H14" s="18" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.15">
+      <c r="B15" s="14">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C15" s="28">
+      <c r="C15" s="22">
         <f>'Step 2'!C15</f>
         <v>0</v>
       </c>
-      <c r="D15" s="31">
+      <c r="D15" s="25">
         <f>'Step 4 Weighted Calc'!D15</f>
         <v>0</v>
       </c>
-      <c r="E15" s="31">
+      <c r="E15" s="25">
         <f>'Step 4 Weighted Calc'!D15*SUM('Step 4 Weighted Calc'!H15:S15)</f>
         <v>0</v>
       </c>
-      <c r="G15" s="21" t="s">
-        <v>6</v>
-      </c>
-      <c r="H15" s="21" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B16" s="16">
+      <c r="G15" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="H15" s="18" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8" x14ac:dyDescent="0.15">
+      <c r="B16" s="14">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C16" s="28">
+      <c r="C16" s="22">
         <f>'Step 2'!C16</f>
         <v>0</v>
       </c>
-      <c r="D16" s="31">
+      <c r="D16" s="25">
         <f>'Step 4 Weighted Calc'!D16</f>
         <v>0</v>
       </c>
-      <c r="E16" s="31">
+      <c r="E16" s="25">
         <f>'Step 4 Weighted Calc'!D16*SUM('Step 4 Weighted Calc'!H16:S16)</f>
         <v>0</v>
       </c>
-      <c r="G16" s="21" t="s">
-        <v>6</v>
-      </c>
-      <c r="H16" s="21" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B17" s="16">
+      <c r="G16" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="H16" s="18" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.15">
+      <c r="B17" s="14">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C17" s="28">
+      <c r="C17" s="22">
         <f>'Step 2'!C17</f>
         <v>0</v>
       </c>
-      <c r="D17" s="31">
+      <c r="D17" s="25">
         <f>'Step 4 Weighted Calc'!D17</f>
         <v>0</v>
       </c>
-      <c r="E17" s="31">
+      <c r="E17" s="25">
         <f>'Step 4 Weighted Calc'!D17*SUM('Step 4 Weighted Calc'!H17:S17)</f>
         <v>0</v>
       </c>
-      <c r="G17" s="21" t="s">
-        <v>6</v>
-      </c>
-      <c r="H17" s="21" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="24" spans="2:8" ht="12" x14ac:dyDescent="0.4">
+      <c r="G17" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="H17" s="18" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.15">
+      <c r="B18" s="14">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="C18" s="22">
+        <f>'Step 2'!C18</f>
+        <v>0</v>
+      </c>
+      <c r="D18" s="25">
+        <f>'Step 4 Weighted Calc'!D18</f>
+        <v>0</v>
+      </c>
+      <c r="E18" s="25">
+        <f>'Step 4 Weighted Calc'!D18*SUM('Step 4 Weighted Calc'!H18:S18)</f>
+        <v>0</v>
+      </c>
+      <c r="G18" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="H18" s="18" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8" ht="14" x14ac:dyDescent="0.3">
       <c r="B24" s="3" t="s">
         <v>122</v>
       </c>
@@ -3667,29 +3812,29 @@
         <v>119</v>
       </c>
     </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:8" x14ac:dyDescent="0.15">
       <c r="C25" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="D25" s="33">
+      <c r="D25" s="26">
         <v>100</v>
       </c>
     </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="C26" s="32" t="str">
+    <row r="26" spans="2:8" x14ac:dyDescent="0.15">
+      <c r="C26" s="3" t="str">
         <f>'Step 4 Weighted Calc'!$C$21</f>
         <v>Today Low</v>
       </c>
-      <c r="D26" s="34">
+      <c r="D26" s="27">
         <f>SUM(E7:E21)*D25</f>
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="C27" s="13" t="s">
+    <row r="27" spans="2:8" x14ac:dyDescent="0.15">
+      <c r="C27" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="D27" s="35">
+      <c r="D27" s="28">
         <f>D25-D26</f>
         <v>100</v>
       </c>
@@ -3702,7 +3847,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{479BF79B-2831-430A-9E0C-CBF400C41427}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3711,464 +3856,464 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00A29453-1950-4E33-A2D2-72D89AD41B8B}">
   <dimension ref="A1:K15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="C1" s="24" t="s">
+      <c r="C1" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="D1" s="24" t="s">
+      <c r="D1" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="E1" s="24" t="s">
+      <c r="E1" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="F1" s="24" t="s">
+      <c r="F1" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="G1" s="24" t="s">
+      <c r="G1" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="H1" s="24" t="s">
+      <c r="H1" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="24" t="s">
+      <c r="I1" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="J1" s="24" t="s">
+      <c r="J1" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="K1" s="24" t="s">
+      <c r="K1" s="19" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A2" s="23" t="s">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="23">
+      <c r="B2">
         <v>0.4</v>
       </c>
-      <c r="C2" s="23">
+      <c r="C2">
         <v>0.65</v>
       </c>
-      <c r="D2" s="23">
+      <c r="D2">
         <v>0.6</v>
       </c>
-      <c r="E2" s="23">
+      <c r="E2">
         <v>0.85</v>
       </c>
-      <c r="F2" s="23">
+      <c r="F2">
         <v>0.75</v>
       </c>
-      <c r="G2" s="23">
+      <c r="G2">
         <v>0.95</v>
       </c>
-      <c r="H2" s="23" t="s">
+      <c r="H2" t="s">
         <v>49</v>
       </c>
-      <c r="I2" s="23" t="s">
+      <c r="I2" t="s">
         <v>50</v>
       </c>
-      <c r="J2" s="23" t="s">
+      <c r="J2" t="s">
         <v>51</v>
       </c>
-      <c r="K2" s="23" t="s">
+      <c r="K2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A3" s="23" t="s">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>53</v>
       </c>
-      <c r="B3" s="23">
+      <c r="B3">
         <v>0.45</v>
       </c>
-      <c r="C3" s="23">
+      <c r="C3">
         <v>0.75</v>
       </c>
-      <c r="D3" s="23">
+      <c r="D3">
         <v>0.65</v>
       </c>
-      <c r="E3" s="23">
+      <c r="E3">
         <v>0.9</v>
       </c>
-      <c r="F3" s="23">
+      <c r="F3">
         <v>0.8</v>
       </c>
-      <c r="G3" s="23">
+      <c r="G3">
         <v>0.97</v>
       </c>
-      <c r="H3" s="23" t="s">
+      <c r="H3" t="s">
         <v>54</v>
       </c>
-      <c r="I3" s="23" t="s">
+      <c r="I3" t="s">
         <v>55</v>
       </c>
-      <c r="J3" s="23" t="s">
+      <c r="J3" t="s">
         <v>56</v>
       </c>
-      <c r="K3" s="23" t="s">
+      <c r="K3" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A4" s="23" t="s">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>58</v>
       </c>
-      <c r="B4" s="23">
+      <c r="B4">
         <v>0.25</v>
       </c>
-      <c r="C4" s="23">
+      <c r="C4">
         <v>0.55000000000000004</v>
       </c>
-      <c r="D4" s="23">
+      <c r="D4">
         <v>0.45</v>
       </c>
-      <c r="E4" s="23">
+      <c r="E4">
         <v>0.75</v>
       </c>
-      <c r="F4" s="23">
+      <c r="F4">
         <v>0.6</v>
       </c>
-      <c r="G4" s="23">
+      <c r="G4">
         <v>0.9</v>
       </c>
-      <c r="H4" s="23" t="s">
+      <c r="H4" t="s">
         <v>59</v>
       </c>
-      <c r="I4" s="23" t="s">
+      <c r="I4" t="s">
         <v>60</v>
       </c>
-      <c r="J4" s="23" t="s">
+      <c r="J4" t="s">
         <v>61</v>
       </c>
-      <c r="K4" s="23" t="s">
+      <c r="K4" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A5" s="23" t="s">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>63</v>
       </c>
-      <c r="B5" s="23">
+      <c r="B5">
         <v>0.4</v>
       </c>
-      <c r="C5" s="23">
+      <c r="C5">
         <v>0.7</v>
       </c>
-      <c r="D5" s="23">
+      <c r="D5">
         <v>0.55000000000000004</v>
       </c>
-      <c r="E5" s="23">
+      <c r="E5">
         <v>0.85</v>
       </c>
-      <c r="F5" s="23">
+      <c r="F5">
         <v>0.75</v>
       </c>
-      <c r="G5" s="23">
+      <c r="G5">
         <v>0.95</v>
       </c>
-      <c r="H5" s="23" t="s">
+      <c r="H5" t="s">
         <v>64</v>
       </c>
-      <c r="I5" s="23" t="s">
+      <c r="I5" t="s">
         <v>65</v>
       </c>
-      <c r="J5" s="23" t="s">
+      <c r="J5" t="s">
         <v>66</v>
       </c>
-      <c r="K5" s="23" t="s">
+      <c r="K5" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A6" s="23" t="s">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>68</v>
       </c>
-      <c r="B6" s="23">
+      <c r="B6">
         <v>0.4</v>
       </c>
-      <c r="C6" s="23">
+      <c r="C6">
         <v>0.7</v>
       </c>
-      <c r="D6" s="23">
+      <c r="D6">
         <v>0.55000000000000004</v>
       </c>
-      <c r="E6" s="23">
+      <c r="E6">
         <v>0.85</v>
       </c>
-      <c r="F6" s="23">
+      <c r="F6">
         <v>0.7</v>
       </c>
-      <c r="G6" s="23">
+      <c r="G6">
         <v>0.95</v>
       </c>
-      <c r="H6" s="23" t="s">
+      <c r="H6" t="s">
         <v>69</v>
       </c>
-      <c r="I6" s="23" t="s">
+      <c r="I6" t="s">
         <v>70</v>
       </c>
-      <c r="J6" s="23" t="s">
+      <c r="J6" t="s">
         <v>71</v>
       </c>
-      <c r="K6" s="23" t="s">
+      <c r="K6" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A7" s="23" t="s">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>73</v>
       </c>
-      <c r="B7" s="23">
+      <c r="B7">
         <v>0.1</v>
       </c>
-      <c r="C7" s="23">
+      <c r="C7">
         <v>0.25</v>
       </c>
-      <c r="D7" s="23">
+      <c r="D7">
         <v>0.2</v>
       </c>
-      <c r="E7" s="23">
+      <c r="E7">
         <v>0.45</v>
       </c>
-      <c r="F7" s="23">
+      <c r="F7">
         <v>0.35</v>
       </c>
-      <c r="G7" s="23">
+      <c r="G7">
         <v>0.65</v>
       </c>
-      <c r="H7" s="23" t="s">
+      <c r="H7" t="s">
         <v>74</v>
       </c>
-      <c r="I7" s="23" t="s">
+      <c r="I7" t="s">
         <v>75</v>
       </c>
-      <c r="J7" s="23" t="s">
+      <c r="J7" t="s">
         <v>76</v>
       </c>
-      <c r="K7" s="23" t="s">
+      <c r="K7" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A8" s="23" t="s">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>78</v>
       </c>
-      <c r="B8" s="23">
+      <c r="B8">
         <v>0.4</v>
       </c>
-      <c r="C8" s="23">
+      <c r="C8">
         <v>0.7</v>
       </c>
-      <c r="D8" s="23">
+      <c r="D8">
         <v>0.6</v>
       </c>
-      <c r="E8" s="23">
+      <c r="E8">
         <v>0.85</v>
       </c>
-      <c r="F8" s="23">
+      <c r="F8">
         <v>0.75</v>
       </c>
-      <c r="G8" s="23">
+      <c r="G8">
         <v>0.95</v>
       </c>
-      <c r="H8" s="23" t="s">
+      <c r="H8" t="s">
         <v>79</v>
       </c>
-      <c r="I8" s="23" t="s">
+      <c r="I8" t="s">
         <v>80</v>
       </c>
-      <c r="J8" s="23" t="s">
+      <c r="J8" t="s">
         <v>81</v>
       </c>
-      <c r="K8" s="23" t="s">
+      <c r="K8" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A9" s="23" t="s">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>83</v>
       </c>
-      <c r="B9" s="23">
+      <c r="B9">
         <v>0.1</v>
       </c>
-      <c r="C9" s="23">
+      <c r="C9">
         <v>0.45</v>
       </c>
-      <c r="D9" s="23">
+      <c r="D9">
         <v>0.2</v>
       </c>
-      <c r="E9" s="23">
+      <c r="E9">
         <v>0.6</v>
       </c>
-      <c r="F9" s="23">
+      <c r="F9">
         <v>0.35</v>
       </c>
-      <c r="G9" s="23">
+      <c r="G9">
         <v>0.8</v>
       </c>
-      <c r="H9" s="23" t="s">
+      <c r="H9" t="s">
         <v>84</v>
       </c>
-      <c r="I9" s="23" t="s">
+      <c r="I9" t="s">
         <v>85</v>
       </c>
-      <c r="J9" s="23" t="s">
+      <c r="J9" t="s">
         <v>86</v>
       </c>
-      <c r="K9" s="23" t="s">
+      <c r="K9" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A10" s="23" t="s">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>88</v>
       </c>
-      <c r="B10" s="23">
+      <c r="B10">
         <v>0.15</v>
       </c>
-      <c r="C10" s="23">
+      <c r="C10">
         <v>0.4</v>
       </c>
-      <c r="D10" s="23">
+      <c r="D10">
         <v>0.35</v>
       </c>
-      <c r="E10" s="23">
+      <c r="E10">
         <v>0.65</v>
       </c>
-      <c r="F10" s="23">
+      <c r="F10">
         <v>0.55000000000000004</v>
       </c>
-      <c r="G10" s="23">
+      <c r="G10">
         <v>0.85</v>
       </c>
-      <c r="H10" s="23" t="s">
+      <c r="H10" t="s">
         <v>89</v>
       </c>
-      <c r="I10" s="23" t="s">
+      <c r="I10" t="s">
         <v>90</v>
       </c>
-      <c r="J10" s="23" t="s">
+      <c r="J10" t="s">
         <v>91</v>
       </c>
-      <c r="K10" s="23" t="s">
+      <c r="K10" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A11" s="23" t="s">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>93</v>
       </c>
-      <c r="B11" s="23">
+      <c r="B11">
         <v>0.2</v>
       </c>
-      <c r="C11" s="23">
+      <c r="C11">
         <v>0.45</v>
       </c>
-      <c r="D11" s="23">
+      <c r="D11">
         <v>0.3</v>
       </c>
-      <c r="E11" s="23">
+      <c r="E11">
         <v>0.6</v>
       </c>
-      <c r="F11" s="23">
+      <c r="F11">
         <v>0.45</v>
       </c>
-      <c r="G11" s="23">
+      <c r="G11">
         <v>0.75</v>
       </c>
-      <c r="H11" s="23" t="s">
+      <c r="H11" t="s">
         <v>94</v>
       </c>
-      <c r="I11" s="23" t="s">
+      <c r="I11" t="s">
         <v>95</v>
       </c>
-      <c r="J11" s="23" t="s">
+      <c r="J11" t="s">
         <v>96</v>
       </c>
-      <c r="K11" s="23" t="s">
+      <c r="K11" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A12" s="23" t="s">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>98</v>
       </c>
-      <c r="B12" s="23">
+      <c r="B12">
         <v>0.45</v>
       </c>
-      <c r="C12" s="23">
+      <c r="C12">
         <v>0.75</v>
       </c>
-      <c r="D12" s="23">
+      <c r="D12">
         <v>0.6</v>
       </c>
-      <c r="E12" s="23">
+      <c r="E12">
         <v>0.85</v>
       </c>
-      <c r="F12" s="23">
+      <c r="F12">
         <v>0.75</v>
       </c>
-      <c r="G12" s="23">
+      <c r="G12">
         <v>0.95</v>
       </c>
-      <c r="H12" s="23" t="s">
+      <c r="H12" t="s">
         <v>99</v>
       </c>
-      <c r="I12" s="23" t="s">
+      <c r="I12" t="s">
         <v>100</v>
       </c>
-      <c r="J12" s="23" t="s">
+      <c r="J12" t="s">
         <v>101</v>
       </c>
-      <c r="K12" s="23" t="s">
+      <c r="K12" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A13" s="23" t="s">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>103</v>
       </c>
-      <c r="B13" s="23">
+      <c r="B13">
         <v>0.05</v>
       </c>
-      <c r="C13" s="23">
+      <c r="C13">
         <v>0.15</v>
       </c>
-      <c r="D13" s="23">
+      <c r="D13">
         <v>0.1</v>
       </c>
-      <c r="E13" s="23">
+      <c r="E13">
         <v>0.25</v>
       </c>
-      <c r="F13" s="23">
+      <c r="F13">
         <v>0.2</v>
       </c>
-      <c r="G13" s="23">
+      <c r="G13">
         <v>0.45</v>
       </c>
-      <c r="H13" s="23" t="s">
+      <c r="H13" t="s">
         <v>104</v>
       </c>
-      <c r="I13" s="23" t="s">
+      <c r="I13" t="s">
         <v>105</v>
       </c>
-      <c r="J13" s="23" t="s">
+      <c r="J13" t="s">
         <v>106</v>
       </c>
-      <c r="K13" s="23" t="s">
+      <c r="K13" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B15">
         <v>100</v>
       </c>
@@ -4179,6 +4324,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100643A18D3E9F31A45B94966FE4E00F6DE" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c07939a5679a659e5300e753429923f6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cd4a04a9-136e-4b3f-8d0e-caebf08e72bf" xmlns:ns3="3e2e96c9-fab6-4978-947b-d1b292f2d3c5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="93f1758667c6f091d09988627faa2dc1" ns2:_="" ns3:_="">
     <xsd:import namespace="cd4a04a9-136e-4b3f-8d0e-caebf08e72bf"/>
@@ -4439,15 +4593,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -4460,13 +4605,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C6EEACA0-B11D-4DE9-9F66-6091F0F861F4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7A7AB736-5EF4-40A0-9A18-7C48F41B5F5F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7A7AB736-5EF4-40A0-9A18-7C48F41B5F5F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C6EEACA0-B11D-4DE9-9F66-6091F0F861F4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="cd4a04a9-136e-4b3f-8d0e-caebf08e72bf"/>
+    <ds:schemaRef ds:uri="3e2e96c9-fab6-4978-947b-d1b292f2d3c5"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7786C670-1A1A-4EA6-B547-FC2FD4F13AE5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7786C670-1A1A-4EA6-B547-FC2FD4F13AE5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="cd4a04a9-136e-4b3f-8d0e-caebf08e72bf"/>
+    <ds:schemaRef ds:uri="3e2e96c9-fab6-4978-947b-d1b292f2d3c5"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>